<commit_message>
API Error Consolidated Update 8/5/2026
</commit_message>
<xml_diff>
--- a/Error Inventory/API Error Consolidated List.xlsx
+++ b/Error Inventory/API Error Consolidated List.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\eagnmnwbp130a.usa.dce.usps.gov\VDIProfiles$\fsbtg0\Documents\API Consolidated file to upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usps365-my.sharepoint.com/personal/norman_negron-munoz_usps_gov/Documents/Documents/EMAS API/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A03FF57B-47E3-4436-9AB2-1F81EE5C8058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1D7F6CC-54AD-42C7-B0CB-9E02EA1564DF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="4" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
   </bookViews>
   <sheets>
     <sheet name="General Errors" sheetId="9" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4235" uniqueCount="1045">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4212" uniqueCount="1049">
   <si>
     <t>API</t>
   </si>
@@ -3222,10 +3222,22 @@
     <t>date</t>
   </si>
   <si>
-    <t>Default address: The address you entered was found but more information is needed (such as an apartment, suite, or box number) to match to a specific address.</t>
-  </si>
-  <si>
-    <t>010007</t>
+    <t>codAmountDueSender is required when packageDescription.extraServices includes of one [915, 917]</t>
+  </si>
+  <si>
+    <t>codAmountDueSender, extraServices</t>
+  </si>
+  <si>
+    <t>destinationEntryFacilityType must be one of (DESTINATION_NETWORK_DISTRIBUTION_CENTER, DESTINATION_SECTIONAL_CENTER_FACILITY, DESTINATION_DELIVERY_UNIT, NONE) when enclosedMailClass is MARKETING_MAIL_PARCELS</t>
+  </si>
+  <si>
+    <t>nonProfit must be true to use non-profit rate indicators 'PN' and 'NN'</t>
+  </si>
+  <si>
+    <t>nonProfit is only valid for mailClass 'MARKETING_MAIL_PARCELS'</t>
+  </si>
+  <si>
+    <t>only non-profit rate indicators 'PN' and 'NN' are allowed when nonProfit is true</t>
   </si>
 </sst>
 </file>
@@ -4221,7 +4233,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -4568,13 +4580,13 @@
       <c r="D15" s="10" t="s">
         <v>975</v>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="24">
         <v>160374</v>
       </c>
       <c r="F15" s="33" t="s">
         <v>933</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="11" t="s">
         <v>936</v>
       </c>
     </row>
@@ -4591,13 +4603,13 @@
       <c r="D16" s="10" t="s">
         <v>975</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="24">
         <v>160385</v>
       </c>
       <c r="F16" s="33" t="s">
         <v>994</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="11" t="s">
         <v>995</v>
       </c>
     </row>
@@ -4614,13 +4626,13 @@
       <c r="D17" s="10" t="s">
         <v>975</v>
       </c>
-      <c r="E17" s="17">
+      <c r="E17" s="24">
         <v>160386</v>
       </c>
       <c r="F17" s="33" t="s">
         <v>994</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="10" t="s">
         <v>996</v>
       </c>
     </row>
@@ -4637,7 +4649,7 @@
       <c r="D18" s="10" t="s">
         <v>975</v>
       </c>
-      <c r="E18" s="17">
+      <c r="E18" s="24">
         <v>160387</v>
       </c>
       <c r="F18" s="33" t="s">
@@ -4660,7 +4672,7 @@
       <c r="D19" s="10" t="s">
         <v>975</v>
       </c>
-      <c r="E19" s="17">
+      <c r="E19" s="24">
         <v>160403</v>
       </c>
       <c r="F19" t="s">
@@ -4668,6 +4680,29 @@
       </c>
       <c r="G19" s="2" t="s">
         <v>1017</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="45">
+      <c r="A20" s="10" t="s">
+        <v>882</v>
+      </c>
+      <c r="B20" s="10">
+        <v>401</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>975</v>
+      </c>
+      <c r="E20" s="24">
+        <v>160419</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>840</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>1045</v>
       </c>
     </row>
   </sheetData>
@@ -7249,28 +7284,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="75">
-      <c r="A8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="19">
-        <v>400</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>954</v>
-      </c>
-      <c r="E8" s="27" t="s">
-        <v>1044</v>
-      </c>
-      <c r="F8" s="27" t="s">
-        <v>858</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>1043</v>
-      </c>
+    <row r="8" spans="1:7">
+      <c r="A8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="5"/>
     </row>
     <row r="9" spans="1:7">
       <c r="B9" s="7"/>
@@ -8213,7 +8232,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G244"/>
+  <dimension ref="A1:G241"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -13666,7 +13685,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="238" spans="1:7" ht="30">
+    <row r="238" spans="1:7">
       <c r="A238" s="20" t="s">
         <v>87</v>
       </c>
@@ -13679,14 +13698,14 @@
       <c r="D238" s="21" t="s">
         <v>958</v>
       </c>
-      <c r="E238" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="F238" s="27" t="s">
-        <v>858</v>
-      </c>
-      <c r="G238" s="5" t="s">
-        <v>20</v>
+      <c r="E238" s="17">
+        <v>160418</v>
+      </c>
+      <c r="F238" s="37" t="s">
+        <v>1044</v>
+      </c>
+      <c r="G238" s="2" t="s">
+        <v>1043</v>
       </c>
     </row>
     <row r="239" spans="1:7">
@@ -13702,14 +13721,14 @@
       <c r="D239" s="21" t="s">
         <v>958</v>
       </c>
-      <c r="E239" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="F239" s="27" t="s">
-        <v>855</v>
-      </c>
-      <c r="G239" s="5" t="s">
-        <v>22</v>
+      <c r="E239" s="17">
+        <v>160420</v>
+      </c>
+      <c r="F239" s="17" t="s">
+        <v>765</v>
+      </c>
+      <c r="G239" s="2" t="s">
+        <v>1046</v>
       </c>
     </row>
     <row r="240" spans="1:7">
@@ -13725,14 +13744,14 @@
       <c r="D240" s="21" t="s">
         <v>958</v>
       </c>
-      <c r="E240" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="F240" s="27" t="s">
-        <v>856</v>
-      </c>
-      <c r="G240" s="5" t="s">
-        <v>24</v>
+      <c r="E240" s="17">
+        <v>160421</v>
+      </c>
+      <c r="F240" s="17" t="s">
+        <v>765</v>
+      </c>
+      <c r="G240" s="2" t="s">
+        <v>1047</v>
       </c>
     </row>
     <row r="241" spans="1:7">
@@ -13748,83 +13767,14 @@
       <c r="D241" s="21" t="s">
         <v>958</v>
       </c>
-      <c r="E241" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="F241" s="27" t="s">
-        <v>857</v>
-      </c>
-      <c r="G241" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="242" spans="1:7" ht="30">
-      <c r="A242" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B242" s="20">
-        <v>400</v>
-      </c>
-      <c r="C242" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D242" s="21" t="s">
-        <v>958</v>
-      </c>
-      <c r="E242" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="F242" s="27" t="s">
-        <v>858</v>
-      </c>
-      <c r="G242" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="243" spans="1:7" ht="30">
-      <c r="A243" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B243" s="20">
-        <v>400</v>
-      </c>
-      <c r="C243" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D243" s="21" t="s">
-        <v>958</v>
-      </c>
-      <c r="E243" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="F243" s="27" t="s">
-        <v>858</v>
-      </c>
-      <c r="G243" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="244" spans="1:7" ht="30">
-      <c r="A244" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B244" s="20">
-        <v>400</v>
-      </c>
-      <c r="C244" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D244" s="21" t="s">
-        <v>958</v>
-      </c>
-      <c r="E244" s="27" t="s">
-        <v>1044</v>
-      </c>
-      <c r="F244" s="27" t="s">
-        <v>858</v>
-      </c>
-      <c r="G244" s="5" t="s">
-        <v>1043</v>
+      <c r="E241" s="17">
+        <v>160422</v>
+      </c>
+      <c r="F241" s="17" t="s">
+        <v>765</v>
+      </c>
+      <c r="G241" s="2" t="s">
+        <v>1048</v>
       </c>
     </row>
   </sheetData>
@@ -21260,6 +21210,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD1EFD7F07544F4C8A5DF6ACE5557D0F" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0a46465e297c47d8b88a71685f887e65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9" xmlns:ns3="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4503a5f252426d71f93d44927b16e869" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -21505,29 +21477,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D590CCA9-7961-4660-BBC6-10104A0DDFD4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F11AB0D6-FBA0-4F11-8778-05A9ADBB93A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21547,32 +21523,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D590CCA9-7961-4660-BBC6-10104A0DDFD4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6c9b68e5-0371-4f27-93af-8d15f794dc29}" enabled="1" method="Privileged" siteId="{a01f407a-85cb-4a16-98bb-f28e6384bd28}" removed="0"/>

</xml_diff>